<commit_message>
Updated constants based on the initial ASTRA v2 prototype.
</commit_message>
<xml_diff>
--- a/params/constants.xlsx
+++ b/params/constants.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antho\Documents\GitHub\model2\params\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdd953d6be32cedf/Documents/PSP Active Controls/ASTRA Model 2 Repo/params/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87EAED42-475D-4B6D-825F-7491F9F8CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{87EAED42-475D-4B6D-825F-7491F9F8CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42638B63-DD7C-4BB6-8283-BC23BA71D2E8}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -74,13 +74,13 @@
     <t>Gravity</t>
   </si>
   <si>
-    <t>0.25,0,0;0,1,0;0,0,1</t>
-  </si>
-  <si>
     <t>T</t>
   </si>
   <si>
     <t>Discreate Time Step</t>
+  </si>
+  <si>
+    <t>0.05,0,0;0,0.053,0;0,0,0.053</t>
   </si>
 </sst>
 </file>
@@ -400,9 +400,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -413,67 +413,67 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>0.995</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>0.753</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4">
-        <v>10</v>
+        <v>9.81</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="B5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7">
         <v>0.01</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Shit STILL doesn't work
</commit_message>
<xml_diff>
--- a/params/constants.xlsx
+++ b/params/constants.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdd953d6be32cedf/Documents/PSP Active Controls/ASTRA Model 2 Repo/params/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{87EAED42-475D-4B6D-825F-7491F9F8CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42638B63-DD7C-4BB6-8283-BC23BA71D2E8}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{87EAED42-475D-4B6D-825F-7491F9F8CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36947D9F-9542-430D-A4F7-2B540E6309DE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Value</t>
   </si>
@@ -81,6 +81,15 @@
   </si>
   <si>
     <t>0.05,0,0;0,0.053,0;0,0,0.053</t>
+  </si>
+  <si>
+    <t>mag</t>
+  </si>
+  <si>
+    <t>0;1;0</t>
+  </si>
+  <si>
+    <t>Magnetometer</t>
   </si>
 </sst>
 </file>
@@ -399,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -476,6 +485,17 @@
         <v>13</v>
       </c>
     </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>